<commit_message>
fixed 3D notebook z conversion error
</commit_message>
<xml_diff>
--- a/examples/Newberry/2D/config/newberry_superhot_config.xlsx
+++ b/examples/Newberry/2D/config/newberry_superhot_config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10703"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smello\code\geoPFA\examples\Newberry\2D\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ntaverna/Documents/geoPFA General/geoPFA workshop/geoPFA/examples/Newberry/2D/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD651167-2F56-4A54-BBDF-69078F259657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12281AE2-BA07-D042-95BD-32A46D742DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3630" yWindow="-15240" windowWidth="17280" windowHeight="13080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" r:id="rId1"/>
@@ -283,9 +283,6 @@
     <t>density</t>
   </si>
   <si>
-    <t>epsg:26910</t>
-  </si>
-  <si>
     <t>reservoir</t>
   </si>
   <si>
@@ -299,6 +296,9 @@
   </si>
   <si>
     <t>insulation</t>
+  </si>
+  <si>
+    <t>m-msl</t>
   </si>
 </sst>
 </file>
@@ -645,14 +645,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="16" max="16" width="8.88671875" customWidth="1"/>
+    <col min="16" max="16" width="8.83203125" customWidth="1"/>
     <col min="17" max="17" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -705,7 +705,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>61</v>
       </c>
@@ -752,7 +752,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F3" t="s">
         <v>71</v>
       </c>
@@ -784,7 +784,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F4" t="s">
         <v>74</v>
       </c>
@@ -816,7 +816,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F5" t="s">
         <v>81</v>
       </c>
@@ -848,9 +848,9 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D6">
         <v>0.4</v>
@@ -883,13 +883,13 @@
         <v>26910</v>
       </c>
       <c r="O6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P6" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F7" t="s">
         <v>71</v>
       </c>
@@ -915,13 +915,13 @@
         <v>26910</v>
       </c>
       <c r="O7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F8" t="s">
         <v>81</v>
       </c>
@@ -947,15 +947,15 @@
         <v>26910</v>
       </c>
       <c r="O8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P8" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G9">
         <v>0.249</v>
@@ -970,15 +970,15 @@
         <v>4326</v>
       </c>
       <c r="O9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="C10" t="s">
         <v>89</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="C10" t="s">
-        <v>90</v>
       </c>
       <c r="D10">
         <v>0.2</v>
@@ -1017,7 +1017,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F11" t="s">
         <v>71</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F12" t="s">
         <v>81</v>
       </c>
@@ -1081,7 +1081,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F13" t="s">
         <v>74</v>
       </c>
@@ -1107,7 +1107,7 @@
         <v>26910</v>
       </c>
       <c r="N13" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="O13" t="s">
         <v>69</v>
@@ -1124,15 +1124,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36350C53-10DF-40B8-A514-0EA653A43886}">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.109375" customWidth="1"/>
-    <col min="2" max="2" width="37.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
-    <col min="4" max="4" width="72.44140625" customWidth="1"/>
+    <col min="1" max="1" width="24.1640625" customWidth="1"/>
+    <col min="2" max="2" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5" customWidth="1"/>
+    <col min="4" max="4" width="72.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>17</v>
       </c>
@@ -1146,7 +1146,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1174,7 +1174,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -1216,7 +1216,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
@@ -1230,7 +1230,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -1244,7 +1244,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="58.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>14</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>15</v>
       </c>
@@ -1272,7 +1272,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>7</v>
       </c>
@@ -1286,7 +1286,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>8</v>
       </c>
@@ -1300,7 +1300,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>12</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>25</v>
       </c>
@@ -1328,7 +1328,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
@@ -1342,7 +1342,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>13</v>
       </c>
@@ -1356,7 +1356,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>16</v>
       </c>
@@ -1370,13 +1370,13 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>

</xml_diff>

<commit_message>
added is_3d back into excel config for 2D example
</commit_message>
<xml_diff>
--- a/examples/Newberry/2D/config/newberry_superhot_config.xlsx
+++ b/examples/Newberry/2D/config/newberry_superhot_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ntaverna/Documents/geoPFA General/geoPFA workshop/geoPFA/examples/Newberry/2D/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12281AE2-BA07-D042-95BD-32A46D742DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{412F62AC-5087-A94C-B65C-719C69C41B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="93">
   <si>
     <t>criteria</t>
   </si>
@@ -299,16 +299,29 @@
   </si>
   <si>
     <t>m-msl</t>
+  </si>
+  <si>
+    <t>is_3d</t>
+  </si>
+  <si>
+    <t>yes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -355,7 +368,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -364,6 +377,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -644,15 +658,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="16" max="16" width="8.83203125" customWidth="1"/>
-    <col min="17" max="17" width="14.33203125" customWidth="1"/>
+    <col min="17" max="17" width="8.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -678,34 +692,37 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>61</v>
       </c>
@@ -731,28 +748,31 @@
         <v>64</v>
       </c>
       <c r="I2" t="s">
+        <v>92</v>
+      </c>
+      <c r="J2" t="s">
         <v>65</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>66</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>67</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>68</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>26910</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>69</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F3" t="s">
         <v>71</v>
       </c>
@@ -763,28 +783,31 @@
         <v>72</v>
       </c>
       <c r="I3" t="s">
+        <v>92</v>
+      </c>
+      <c r="J3" t="s">
         <v>73</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>66</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>67</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>68</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>26910</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>69</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F4" t="s">
         <v>74</v>
       </c>
@@ -795,28 +818,31 @@
         <v>75</v>
       </c>
       <c r="I4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J4" t="s">
         <v>76</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>77</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>78</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>79</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>26910</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>80</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F5" t="s">
         <v>81</v>
       </c>
@@ -827,28 +853,31 @@
         <v>82</v>
       </c>
       <c r="I5" t="s">
+        <v>92</v>
+      </c>
+      <c r="J5" t="s">
         <v>83</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>77</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>78</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>79</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>26910</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>69</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
         <v>85</v>
       </c>
@@ -868,28 +897,31 @@
         <v>64</v>
       </c>
       <c r="I6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J6" t="s">
         <v>65</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>66</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>67</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>68</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>26910</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>86</v>
       </c>
-      <c r="P6" t="s">
+      <c r="Q6" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F7" t="s">
         <v>71</v>
       </c>
@@ -900,28 +932,31 @@
         <v>72</v>
       </c>
       <c r="I7" t="s">
+        <v>92</v>
+      </c>
+      <c r="J7" t="s">
         <v>73</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>66</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>67</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>68</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>26910</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>86</v>
       </c>
-      <c r="P7" t="s">
+      <c r="Q7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F8" t="s">
         <v>81</v>
       </c>
@@ -932,28 +967,31 @@
         <v>82</v>
       </c>
       <c r="I8" t="s">
+        <v>92</v>
+      </c>
+      <c r="J8" t="s">
         <v>83</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>77</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>78</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>79</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>26910</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>86</v>
       </c>
-      <c r="P8" t="s">
+      <c r="Q8" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F9" t="s">
         <v>87</v>
       </c>
@@ -963,20 +1001,20 @@
       <c r="H9" t="s">
         <v>80</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>80</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>4326</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>86</v>
       </c>
-      <c r="P9" t="s">
+      <c r="Q9" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="C10" t="s">
         <v>89</v>
       </c>
@@ -995,29 +1033,32 @@
       <c r="H10" t="s">
         <v>64</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J10" t="s">
         <v>65</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>66</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>67</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>68</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <v>26910</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>80</v>
       </c>
-      <c r="P10" t="s">
+      <c r="Q10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F11" t="s">
         <v>71</v>
       </c>
@@ -1027,29 +1068,32 @@
       <c r="H11" t="s">
         <v>72</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J11" t="s">
         <v>73</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>66</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>67</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>68</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>26910</v>
       </c>
-      <c r="O11" t="s">
+      <c r="P11" t="s">
         <v>80</v>
       </c>
-      <c r="P11" t="s">
+      <c r="Q11" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F12" t="s">
         <v>81</v>
       </c>
@@ -1059,29 +1103,32 @@
       <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J12" t="s">
         <v>83</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>77</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>78</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>79</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>26910</v>
       </c>
-      <c r="O12" t="s">
+      <c r="P12" t="s">
         <v>69</v>
       </c>
-      <c r="P12" t="s">
+      <c r="Q12" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F13" t="s">
         <v>74</v>
       </c>
@@ -1091,28 +1138,31 @@
       <c r="H13" t="s">
         <v>75</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J13" t="s">
         <v>76</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>77</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>78</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>79</v>
       </c>
-      <c r="M13">
+      <c r="N13">
         <v>26910</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>90</v>
       </c>
-      <c r="O13" t="s">
+      <c r="P13" t="s">
         <v>69</v>
       </c>
-      <c r="P13" t="s">
+      <c r="Q13" t="s">
         <v>70</v>
       </c>
     </row>

</xml_diff>